<commit_message>
Update default species spreadsheet
- NaturalDeathRate/Variance updated to 0.02/0.01 for all Tier 2/3 species
- Added Common Values reference table
- Added NaturalDeathRate/Variance columns to mortality table
</commit_message>
<xml_diff>
--- a/Default species.xlsx
+++ b/Default species.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Work Projects\TinySea\tinysea\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D360578-2789-40E5-A34A-698F940EF27F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92A4E31D-ABF7-4404-84F9-043B2E577F75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="123">
   <si>
     <t>Index</t>
   </si>
@@ -311,6 +311,15 @@
     <t>Thermal Limits &amp; Performance by Variant</t>
   </si>
   <si>
+    <t>Common Values (All Species)</t>
+  </si>
+  <si>
+    <t>Parameter</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
     <t>Common (Generalist)</t>
   </si>
   <si>
@@ -330,12 +339,6 @@
   </si>
   <si>
     <t>Default Simulation Config</t>
-  </si>
-  <si>
-    <t>Parameter</t>
-  </si>
-  <si>
-    <t>Value</t>
   </si>
   <si>
     <t>BiologyStep</t>
@@ -396,7 +399,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.############"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -412,6 +415,16 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -463,7 +476,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -648,26 +661,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -799,16 +797,38 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3388,10 +3408,10 @@
         <v>0</v>
       </c>
       <c r="AC11">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD11">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE11">
         <v>0.75</v>
@@ -3487,10 +3507,10 @@
         <v>0</v>
       </c>
       <c r="AC12">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD12">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE12">
         <v>0.75</v>
@@ -3586,10 +3606,10 @@
         <v>0</v>
       </c>
       <c r="AC13">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD13">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE13">
         <v>0.75</v>
@@ -3685,10 +3705,10 @@
         <v>0</v>
       </c>
       <c r="AC14">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD14">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE14">
         <v>0.75</v>
@@ -3784,10 +3804,10 @@
         <v>0</v>
       </c>
       <c r="AC15">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD15">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE15">
         <v>0.75</v>
@@ -3883,10 +3903,10 @@
         <v>0</v>
       </c>
       <c r="AC16">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD16">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE16">
         <v>0.75</v>
@@ -3982,10 +4002,10 @@
         <v>0</v>
       </c>
       <c r="AC17">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD17">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE17">
         <v>0.75</v>
@@ -4081,10 +4101,10 @@
         <v>0</v>
       </c>
       <c r="AC18">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD18">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE18">
         <v>0.75</v>
@@ -4180,10 +4200,10 @@
         <v>0</v>
       </c>
       <c r="AC19">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD19">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE19">
         <v>0.75</v>
@@ -4279,10 +4299,10 @@
         <v>0</v>
       </c>
       <c r="AC20">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD20">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE20">
         <v>0.75</v>
@@ -4378,10 +4398,10 @@
         <v>0</v>
       </c>
       <c r="AC21">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD21">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE21">
         <v>0.75</v>
@@ -4477,10 +4497,10 @@
         <v>0</v>
       </c>
       <c r="AC22">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD22">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE22">
         <v>0.75</v>
@@ -4576,10 +4596,10 @@
         <v>0</v>
       </c>
       <c r="AC23">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD23">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE23">
         <v>0.75</v>
@@ -4675,10 +4695,10 @@
         <v>0</v>
       </c>
       <c r="AC24">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD24">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE24">
         <v>0.75</v>
@@ -4774,10 +4794,10 @@
         <v>0</v>
       </c>
       <c r="AC25">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD25">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE25">
         <v>0.75</v>
@@ -4873,10 +4893,10 @@
         <v>0</v>
       </c>
       <c r="AC26">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD26">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE26">
         <v>0.75</v>
@@ -4972,10 +4992,10 @@
         <v>0</v>
       </c>
       <c r="AC27">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD27">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE27">
         <v>0.75</v>
@@ -5071,10 +5091,10 @@
         <v>0</v>
       </c>
       <c r="AC28" s="25">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AD28" s="25">
-        <v>1.4999999999999999E-2</v>
+        <v>0.01</v>
       </c>
       <c r="AE28" s="25">
         <v>0.75</v>
@@ -5121,7 +5141,6 @@
       <c r="G30" s="42"/>
       <c r="H30" s="42"/>
       <c r="I30" s="43"/>
-      <c r="M30" s="2"/>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" s="2"/>
@@ -5149,7 +5168,6 @@
       <c r="I31" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="M31" s="2"/>
       <c r="N31" s="2"/>
       <c r="O31" s="2"/>
       <c r="P31" s="2"/>
@@ -5166,7 +5184,7 @@
     <row r="32" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C32" s="2"/>
       <c r="F32" s="31" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="G32" s="27">
         <v>0.9</v>
@@ -5177,7 +5195,6 @@
       <c r="I32" s="32">
         <v>40</v>
       </c>
-      <c r="M32" s="2"/>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
       <c r="P32" s="2"/>
@@ -5194,7 +5211,7 @@
     <row r="33" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C33" s="2"/>
       <c r="F33" s="31" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="G33" s="27">
         <v>1</v>
@@ -5205,7 +5222,6 @@
       <c r="I33" s="32">
         <v>80</v>
       </c>
-      <c r="M33" s="2"/>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
       <c r="P33" s="2"/>
@@ -5222,7 +5238,7 @@
     <row r="34" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C34" s="2"/>
       <c r="F34" s="33" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="G34" s="34">
         <v>1</v>
@@ -5233,7 +5249,6 @@
       <c r="I34" s="35">
         <v>20</v>
       </c>
-      <c r="M34" s="2"/>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
       <c r="P34" s="2"/>
@@ -5259,8 +5274,6 @@
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
       <c r="K35" s="2"/>
-      <c r="L35" s="2"/>
-      <c r="M35" s="2"/>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" s="2"/>
@@ -5279,12 +5292,12 @@
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
       <c r="F36" s="44" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="G36" s="45"/>
       <c r="H36" s="46"/>
-      <c r="I36" s="50"/>
-      <c r="J36" s="50"/>
+      <c r="I36" s="1"/>
+      <c r="J36" s="1"/>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" s="2"/>
@@ -5308,6 +5321,8 @@
       <c r="H37" s="38" t="s">
         <v>31</v>
       </c>
+      <c r="I37" s="47"/>
+      <c r="J37" s="47"/>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
       <c r="P37" s="2"/>
@@ -5323,7 +5338,7 @@
     </row>
     <row r="38" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="F38" s="39" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="G38" s="1" t="s">
         <v>35</v>
@@ -5346,7 +5361,7 @@
     </row>
     <row r="39" spans="1:33" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="F39" s="40" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="G39" s="22">
         <v>0.75</v>
@@ -5393,10 +5408,10 @@
       <c r="A41" s="2"/>
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
-      <c r="F41" s="49" t="s">
-        <v>102</v>
-      </c>
-      <c r="G41" s="46"/>
+      <c r="F41" s="55" t="s">
+        <v>105</v>
+      </c>
+      <c r="G41" s="56"/>
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
@@ -5420,11 +5435,11 @@
       <c r="A42" s="2"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
-      <c r="F42" s="47" t="s">
-        <v>103</v>
-      </c>
-      <c r="G42" s="47" t="s">
-        <v>104</v>
+      <c r="F42" s="57" t="s">
+        <v>97</v>
+      </c>
+      <c r="G42" s="58" t="s">
+        <v>98</v>
       </c>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
@@ -5449,10 +5464,10 @@
       <c r="A43" s="2"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
-      <c r="F43" s="48" t="s">
-        <v>105</v>
-      </c>
-      <c r="G43" s="48">
+      <c r="F43" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="G43" s="20">
         <v>1</v>
       </c>
       <c r="H43" s="2"/>
@@ -5478,10 +5493,10 @@
       <c r="A44" s="2"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
-      <c r="F44" s="48" t="s">
-        <v>106</v>
-      </c>
-      <c r="G44" s="48">
+      <c r="F44" s="39" t="s">
+        <v>107</v>
+      </c>
+      <c r="G44" s="20">
         <v>365</v>
       </c>
       <c r="H44" s="2"/>
@@ -5507,10 +5522,10 @@
       <c r="A45" s="2"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
-      <c r="F45" s="48" t="s">
-        <v>107</v>
-      </c>
-      <c r="G45" s="48">
+      <c r="F45" s="39" t="s">
+        <v>108</v>
+      </c>
+      <c r="G45" s="20">
         <v>5</v>
       </c>
       <c r="H45" s="2"/>
@@ -5536,10 +5551,10 @@
       <c r="A46" s="2"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
-      <c r="F46" s="48" t="s">
-        <v>108</v>
-      </c>
-      <c r="G46" s="48" t="b">
+      <c r="F46" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="G46" s="20" t="b">
         <v>1</v>
       </c>
       <c r="H46" s="2"/>
@@ -5565,10 +5580,10 @@
       <c r="A47" s="2"/>
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
-      <c r="F47" s="48" t="s">
-        <v>109</v>
-      </c>
-      <c r="G47" s="48">
+      <c r="F47" s="39" t="s">
+        <v>110</v>
+      </c>
+      <c r="G47" s="20">
         <v>5000</v>
       </c>
       <c r="H47" s="2"/>
@@ -5594,10 +5609,10 @@
       <c r="A48" s="2"/>
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
-      <c r="F48" s="48" t="s">
-        <v>110</v>
-      </c>
-      <c r="G48" s="48">
+      <c r="F48" s="39" t="s">
+        <v>111</v>
+      </c>
+      <c r="G48" s="20">
         <v>20</v>
       </c>
       <c r="H48" s="2"/>
@@ -5623,10 +5638,10 @@
       <c r="A49" s="2"/>
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
-      <c r="F49" s="48" t="s">
-        <v>111</v>
-      </c>
-      <c r="G49" s="48">
+      <c r="F49" s="39" t="s">
+        <v>112</v>
+      </c>
+      <c r="G49" s="20">
         <v>10</v>
       </c>
       <c r="H49" s="2"/>
@@ -5652,10 +5667,10 @@
       <c r="A50" s="2"/>
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
-      <c r="F50" s="48" t="s">
-        <v>112</v>
-      </c>
-      <c r="G50" s="48">
+      <c r="F50" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="G50" s="20">
         <v>1</v>
       </c>
       <c r="H50" s="2"/>
@@ -5681,10 +5696,10 @@
       <c r="A51" s="2"/>
       <c r="B51" s="1"/>
       <c r="C51" s="1"/>
-      <c r="F51" s="48" t="s">
-        <v>113</v>
-      </c>
-      <c r="G51" s="48" t="b">
+      <c r="F51" s="39" t="s">
+        <v>114</v>
+      </c>
+      <c r="G51" s="20" t="b">
         <v>1</v>
       </c>
       <c r="H51" s="2"/>
@@ -5710,10 +5725,10 @@
       <c r="A52" s="2"/>
       <c r="B52" s="1"/>
       <c r="C52" s="1"/>
-      <c r="F52" s="48" t="s">
-        <v>114</v>
-      </c>
-      <c r="G52" s="48">
+      <c r="F52" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="G52" s="20">
         <v>2</v>
       </c>
       <c r="H52" s="2"/>
@@ -5739,10 +5754,10 @@
       <c r="A53" s="2"/>
       <c r="B53" s="1"/>
       <c r="C53" s="1"/>
-      <c r="F53" s="48" t="s">
-        <v>115</v>
-      </c>
-      <c r="G53" s="48">
+      <c r="F53" s="39" t="s">
+        <v>116</v>
+      </c>
+      <c r="G53" s="20">
         <v>1.5</v>
       </c>
       <c r="H53" s="2"/>
@@ -5768,10 +5783,10 @@
       <c r="A54" s="2"/>
       <c r="B54" s="1"/>
       <c r="C54" s="1"/>
-      <c r="F54" s="48" t="s">
-        <v>116</v>
-      </c>
-      <c r="G54" s="48" t="b">
+      <c r="F54" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="G54" s="20" t="b">
         <v>1</v>
       </c>
       <c r="H54" s="2"/>
@@ -5797,10 +5812,10 @@
       <c r="A55" s="2"/>
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
-      <c r="F55" s="48" t="s">
-        <v>117</v>
-      </c>
-      <c r="G55" s="48">
+      <c r="F55" s="39" t="s">
+        <v>118</v>
+      </c>
+      <c r="G55" s="20">
         <v>5</v>
       </c>
       <c r="H55" s="2"/>
@@ -5826,10 +5841,10 @@
       <c r="A56" s="2"/>
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
-      <c r="F56" s="48" t="s">
-        <v>118</v>
-      </c>
-      <c r="G56" s="48">
+      <c r="F56" s="39" t="s">
+        <v>119</v>
+      </c>
+      <c r="G56" s="20">
         <v>0.5</v>
       </c>
       <c r="H56" s="2"/>
@@ -5855,10 +5870,10 @@
       <c r="A57" s="2"/>
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
-      <c r="F57" s="48" t="s">
-        <v>119</v>
-      </c>
-      <c r="G57" s="48">
+      <c r="F57" s="39" t="s">
+        <v>120</v>
+      </c>
+      <c r="G57" s="20">
         <v>-5</v>
       </c>
       <c r="H57" s="2"/>
@@ -5884,10 +5899,10 @@
       <c r="A58" s="2"/>
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
-      <c r="F58" s="48" t="s">
-        <v>120</v>
-      </c>
-      <c r="G58" s="48">
+      <c r="F58" s="39" t="s">
+        <v>121</v>
+      </c>
+      <c r="G58" s="20">
         <v>50</v>
       </c>
       <c r="H58" s="2"/>
@@ -5913,10 +5928,10 @@
       <c r="A59" s="2"/>
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
-      <c r="F59" s="48" t="s">
-        <v>121</v>
-      </c>
-      <c r="G59" s="48">
+      <c r="F59" s="40" t="s">
+        <v>122</v>
+      </c>
+      <c r="G59" s="26">
         <v>12345</v>
       </c>
       <c r="H59" s="2"/>
@@ -5969,8 +5984,10 @@
       <c r="C61" s="1"/>
       <c r="D61" s="2"/>
       <c r="E61" s="2"/>
-      <c r="F61" s="2"/>
-      <c r="G61" s="2"/>
+      <c r="F61" s="54" t="s">
+        <v>96</v>
+      </c>
+      <c r="G61" s="46"/>
       <c r="H61" s="2"/>
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
@@ -5996,8 +6013,12 @@
       <c r="C62" s="1"/>
       <c r="D62" s="2"/>
       <c r="E62" s="2"/>
-      <c r="F62" s="2"/>
-      <c r="G62" s="2"/>
+      <c r="F62" s="48" t="s">
+        <v>97</v>
+      </c>
+      <c r="G62" s="49" t="s">
+        <v>98</v>
+      </c>
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
@@ -6023,8 +6044,12 @@
       <c r="C63" s="1"/>
       <c r="D63" s="2"/>
       <c r="E63" s="2"/>
-      <c r="F63" s="2"/>
-      <c r="G63" s="2"/>
+      <c r="F63" s="50" t="s">
+        <v>7</v>
+      </c>
+      <c r="G63" s="20">
+        <v>0.3</v>
+      </c>
       <c r="H63" s="2"/>
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
@@ -6050,8 +6075,12 @@
       <c r="C64" s="1"/>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
-      <c r="F64" s="2"/>
-      <c r="G64" s="2"/>
+      <c r="F64" s="50" t="s">
+        <v>9</v>
+      </c>
+      <c r="G64" s="20">
+        <v>1</v>
+      </c>
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
@@ -6077,8 +6106,12 @@
       <c r="C65" s="1"/>
       <c r="D65" s="2"/>
       <c r="E65" s="2"/>
-      <c r="F65" s="2"/>
-      <c r="G65" s="2"/>
+      <c r="F65" s="50" t="s">
+        <v>10</v>
+      </c>
+      <c r="G65" s="20">
+        <v>0.25</v>
+      </c>
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
@@ -6104,8 +6137,12 @@
       <c r="C66" s="1"/>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
-      <c r="F66" s="2"/>
-      <c r="G66" s="2"/>
+      <c r="F66" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="G66" s="20">
+        <v>0.02</v>
+      </c>
       <c r="H66" s="2"/>
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
@@ -6131,8 +6168,12 @@
       <c r="C67" s="1"/>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
-      <c r="F67" s="2"/>
-      <c r="G67" s="2"/>
+      <c r="F67" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="G67" s="51">
+        <v>0.01</v>
+      </c>
       <c r="H67" s="2"/>
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
@@ -6158,8 +6199,12 @@
       <c r="C68" s="1"/>
       <c r="D68" s="2"/>
       <c r="E68" s="2"/>
-      <c r="F68" s="2"/>
-      <c r="G68" s="2"/>
+      <c r="F68" s="52" t="s">
+        <v>27</v>
+      </c>
+      <c r="G68" s="53">
+        <v>0</v>
+      </c>
       <c r="H68" s="2"/>
       <c r="I68" s="2"/>
       <c r="J68" s="2"/>
@@ -31344,7 +31389,7 @@
       <c r="AG1000" s="4"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D1:D29 I30:I34 D35 F41:F60 D61:D1000 I36 G37:G39">
+  <conditionalFormatting sqref="D1:D29 I30:I34 D35 I36 G37:G39 F41:F60 D61:D1000">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Arctic"</formula>
     </cfRule>

</xml_diff>